<commit_message>
Updated Spring Backlog time
Added Time for Development with Grade class.
</commit_message>
<xml_diff>
--- a/documentation/Sprint Backlog Burndown.xlsx
+++ b/documentation/Sprint Backlog Burndown.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrocker1\Desktop\DevOps\Project\DevOps-F26-Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF16872E-18EF-4A41-8679-E80DB6E9A7B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{992214CB-F7A4-44D9-BB4F-4123AF7964F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="1520" windowWidth="25580" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -362,7 +362,7 @@
                   <c:v>16.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>4.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1493,7 +1493,9 @@
       <c r="C5" s="1">
         <v>2</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2">
+        <v>0.5</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1523,7 +1525,9 @@
       <c r="C7" s="1">
         <v>1</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2">
+        <v>3</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1551,7 +1555,9 @@
       <c r="C9" s="1">
         <v>2</v>
       </c>
-      <c r="D9" s="2"/>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1776,7 +1782,7 @@
       </c>
       <c r="D30" s="3">
         <f>SUM(D3:D29)</f>
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="E30" s="3">
         <f>SUM(E3:E29)</f>

</xml_diff>

<commit_message>
Updated Sprint Backlog Hours
Updated Hours to reflect time spent working on Grade and Subsection implementation.
</commit_message>
<xml_diff>
--- a/documentation/Sprint Backlog Burndown.xlsx
+++ b/documentation/Sprint Backlog Burndown.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrocker1\Desktop\DevOps\Project\DevOps-F26-Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{992214CB-F7A4-44D9-BB4F-4123AF7964F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615FF5F5-ABE2-4729-B738-2F086DD499BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -362,10 +362,10 @@
                   <c:v>16.25</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.5</c:v>
+                  <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1414,14 +1414,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="2" width="50.26953125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1438,7 +1438,7 @@
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="10"/>
       <c r="B2" s="11"/>
       <c r="C2" s="10"/>
@@ -1455,7 +1455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -1470,7 +1470,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>
       <c r="B4" s="6" t="s">
         <v>20</v>
@@ -1483,7 +1483,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>25</v>
       </c>
@@ -1500,7 +1500,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1515,7 +1515,7 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
@@ -1528,11 +1528,13 @@
       <c r="D7" s="2">
         <v>3</v>
       </c>
-      <c r="E7" s="2"/>
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="6" t="s">
         <v>17</v>
@@ -1541,11 +1543,13 @@
         <v>2</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="E8" s="2">
+        <v>2</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1556,13 +1560,15 @@
         <v>2</v>
       </c>
       <c r="D9" s="2">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2">
         <v>1</v>
       </c>
-      <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1577,7 +1583,7 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>11</v>
       </c>
@@ -1592,7 +1598,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1602,12 +1608,14 @@
       <c r="C12" s="1">
         <v>1</v>
       </c>
-      <c r="D12" s="2"/>
+      <c r="D12" s="2">
+        <v>1</v>
+      </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
@@ -1622,7 +1630,7 @@
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
@@ -1637,7 +1645,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
       <c r="C15" s="1"/>
@@ -1646,7 +1654,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
       <c r="C16" s="1"/>
@@ -1655,7 +1663,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
       <c r="C17" s="1"/>
@@ -1664,7 +1672,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
       <c r="C18" s="1"/>
@@ -1673,7 +1681,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
       <c r="C19" s="1"/>
@@ -1682,7 +1690,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
       <c r="C20" s="1"/>
@@ -1691,7 +1699,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
       <c r="B21" s="6"/>
       <c r="C21" s="1"/>
@@ -1700,7 +1708,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="6"/>
       <c r="C22" s="1"/>
@@ -1709,7 +1717,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="6"/>
       <c r="C23" s="1"/>
@@ -1718,7 +1726,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
       <c r="B24" s="6"/>
       <c r="C24" s="1"/>
@@ -1727,7 +1735,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
       <c r="B25" s="6"/>
       <c r="C25" s="1"/>
@@ -1736,7 +1744,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
       <c r="B26" s="6"/>
       <c r="C26" s="1"/>
@@ -1745,7 +1753,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
       <c r="B27" s="6"/>
       <c r="C27" s="1"/>
@@ -1754,7 +1762,7 @@
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
       <c r="B28" s="6"/>
       <c r="C28" s="1"/>
@@ -1763,7 +1771,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
       <c r="B29" s="6"/>
       <c r="C29" s="1"/>
@@ -1772,7 +1780,7 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">
         <v>8</v>
       </c>
@@ -1782,11 +1790,11 @@
       </c>
       <c r="D30" s="3">
         <f>SUM(D3:D29)</f>
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="E30" s="3">
         <f>SUM(E3:E29)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F30" s="3">
         <f>SUM(F3:F29)</f>
@@ -1797,27 +1805,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>35</v>
       </c>

</xml_diff>

<commit_message>
Implemented Displaying Course Info
Implemented displaying the course data to the CourseSelectionWindow. Formatted the Average and End Grade to be only two digits after the decimal point.
Implemented Course to get the Average and End grade of a Course.
Fixed some logic with getting the End Grade, used getScore instead of getPercentage and it messed with the average of the points.
Added Tests to test for classes that don't have 100 as the Max points to verify it works properly.
</commit_message>
<xml_diff>
--- a/documentation/Sprint Backlog Burndown.xlsx
+++ b/documentation/Sprint Backlog Burndown.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrocker1\Desktop\DevOps\Project\DevOps-F26-Project\documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615FF5F5-ABE2-4729-B738-2F086DD499BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A522706-1DFE-4A88-BFAA-B3AF6BB27987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Related User Story</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>SubSections has Name, Weight, and # of Assignments (Optional?)</t>
+  </si>
+  <si>
+    <t>Worked on 10/10 from 11AM to 3:30 and from 9PM to 2 AM</t>
   </si>
 </sst>
 </file>
@@ -365,7 +368,7 @@
                   <c:v>6.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1413,15 +1416,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
-    <col min="2" max="2" width="50.28515625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="50.26953125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1438,7 +1441,7 @@
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="10"/>
       <c r="B2" s="11"/>
       <c r="C2" s="10"/>
@@ -1455,7 +1458,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
         <v>18</v>
       </c>
@@ -1466,11 +1469,13 @@
         <v>1.5</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2">
+        <v>2</v>
+      </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="5"/>
       <c r="B4" s="6" t="s">
         <v>20</v>
@@ -1479,11 +1484,13 @@
         <v>2</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="E4" s="2">
+        <v>2</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>25</v>
       </c>
@@ -1496,11 +1503,13 @@
       <c r="D5" s="2">
         <v>0.5</v>
       </c>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2">
+        <v>2</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -1511,11 +1520,13 @@
         <v>1</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="E6" s="2">
+        <v>2</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
@@ -1534,7 +1545,7 @@
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" s="5"/>
       <c r="B8" s="6" t="s">
         <v>17</v>
@@ -1549,7 +1560,7 @@
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -1563,12 +1574,12 @@
         <v>2</v>
       </c>
       <c r="E9" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -1583,7 +1594,7 @@
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>11</v>
       </c>
@@ -1598,7 +1609,7 @@
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>12</v>
       </c>
@@ -1611,11 +1622,13 @@
       <c r="D12" s="2">
         <v>1</v>
       </c>
-      <c r="E12" s="2"/>
+      <c r="E12" s="2">
+        <v>1</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
@@ -1626,11 +1639,13 @@
         <v>0.25</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2">
+        <v>1</v>
+      </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
     </row>
-    <row r="14" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
@@ -1645,7 +1660,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="6"/>
       <c r="C15" s="1"/>
@@ -1654,7 +1669,7 @@
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="6"/>
       <c r="C16" s="1"/>
@@ -1663,7 +1678,7 @@
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="6"/>
       <c r="C17" s="1"/>
@@ -1672,7 +1687,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="6"/>
       <c r="C18" s="1"/>
@@ -1681,7 +1696,7 @@
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="6"/>
       <c r="C19" s="1"/>
@@ -1690,7 +1705,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="6"/>
       <c r="C20" s="1"/>
@@ -1699,7 +1714,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="6"/>
       <c r="C21" s="1"/>
@@ -1708,7 +1723,7 @@
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="6"/>
       <c r="C22" s="1"/>
@@ -1717,7 +1732,7 @@
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="6"/>
       <c r="C23" s="1"/>
@@ -1726,7 +1741,7 @@
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="6"/>
       <c r="C24" s="1"/>
@@ -1735,7 +1750,7 @@
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="6"/>
       <c r="C25" s="1"/>
@@ -1744,7 +1759,7 @@
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="6"/>
       <c r="C26" s="1"/>
@@ -1753,7 +1768,7 @@
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="6"/>
       <c r="C27" s="1"/>
@@ -1762,7 +1777,7 @@
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="6"/>
       <c r="C28" s="1"/>
@@ -1771,7 +1786,7 @@
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="6"/>
       <c r="C29" s="1"/>
@@ -1780,7 +1795,7 @@
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B30" s="7" t="s">
         <v>8</v>
       </c>
@@ -1794,7 +1809,7 @@
       </c>
       <c r="E30" s="3">
         <f>SUM(E3:E29)</f>
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F30" s="3">
         <f>SUM(F3:F29)</f>
@@ -1805,29 +1820,34 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>